<commit_message>
Update NLP documentation and Feature Contract Matrix for the four-class classifier
- CLAUDE.md: NLP/SVM is in scope (RQ2); doctor-only, not stored, English-only
  support claim; not yet deployed or tested end to end.
- NLP.md, NLP_RESEARCH_ALIGNMENT.md: final dataset is 500 texts (v1.0);
  dataset languages vs claimed English-only support.
- NLP_WORK_LOG.md: dated entry for Oct 9-13.
- BACKEND_Implementation.md: language and storage decisions; frontend wiring.
- Feature Contract Matrix: add PStress1 row (Partial; testing pending).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6QEi5po5r8gdN2M1jsjBX
</commit_message>
<xml_diff>
--- a/VitalSync - FeatureContractMatrix.xlsx
+++ b/VitalSync - FeatureContractMatrix.xlsx
@@ -2121,19 +2121,76 @@
       </c>
     </row>
     <row r="24" ht="60.0" customHeight="1">
-      <c r="A24" s="37"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="39"/>
-      <c r="L24" s="39"/>
-      <c r="M24" s="39"/>
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PStress1</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stress classification (SVM)</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patient → Doctor</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sees the four-class stress classification (No/Mild/Moderate/High Stress) of the patient's latest stress reflection in the doctor-side Your Journey</t>
+        </is>
+      </c>
+      <c r="E24" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submits a stress reflection (Express Yourself or Guided Reflection with the five final questions). Does not see the classification</t>
+        </is>
+      </c>
+      <c r="F24" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠️ Partial</t>
+        </is>
+      </c>
+      <c r="G24" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doctor + Backend</t>
+        </is>
+      </c>
+      <c r="H24" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stress</t>
+        </is>
+      </c>
+      <c r="I24" s="35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🔴 HIGH</t>
+        </is>
+      </c>
+      <c r="J24" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Doctor-only. Not a diagnosis, score or treatment recommendation
+- Result returned on request, not stored
+- Input: non-empty answers in Q1–Q5 order, joined with single spaces; all blank → unable to classify
+- Social and Habits reflections are not classified
+- Support claimed for English only
+- Endpoint POST /api/patients/&lt;id&gt;/stress-classification not yet deployed; end-to-end test pending</t>
+        </is>
+      </c>
+      <c r="K24" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✅</t>
+        </is>
+      </c>
+      <c r="L24" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✅</t>
+        </is>
+      </c>
+      <c r="M24" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">❌</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="60.0" customHeight="1">
       <c r="A25" s="37"/>

</xml_diff>

<commit_message>
Mark PStress1 workflow complete
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/VitalSync - FeatureContractMatrix.xlsx
+++ b/VitalSync - FeatureContractMatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesiah\Desktop\Teyvat\Coding\3rdYear\SIA2\VitalSyncPrototype\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE804C37-FD10-4694-A3DE-022DB7D5C45A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DD12F3-2193-42F9-9230-FA9474A8DBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feature Contract Matrix" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="155">
   <si>
     <t>Idea</t>
   </si>
@@ -543,6 +543,9 @@
 - Social and Habits reflections are not classified
 - Support claimed for English only
 - Merged to main (b6321bc) and deployed. E2E-01–19 passed on the isolated test setup (Oct 14–15); post-merge E2E-01/12/13 passed on the production setup (Oct 19).</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -2231,10 +2234,10 @@
         <v>151</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>50</v>
+        <v>154</v>
       </c>
       <c r="H24" s="29" t="s">
         <v>152</v>

</xml_diff>

<commit_message>
updated "PStress1" in VitalSync - FeatureContractMatrix
</commit_message>
<xml_diff>
--- a/VitalSync - FeatureContractMatrix.xlsx
+++ b/VitalSync - FeatureContractMatrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesiah\Desktop\Teyvat\Coding\3rdYear\SIA2\VitalSyncPrototype\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DD12F3-2193-42F9-9230-FA9474A8DBF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC5DB51-E9AB-47F9-8D99-0E627B1589E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="154">
   <si>
     <t>Idea</t>
   </si>
@@ -543,9 +543,6 @@
 - Social and Habits reflections are not classified
 - Support claimed for English only
 - Merged to main (b6321bc) and deployed. E2E-01–19 passed on the isolated test setup (Oct 14–15); post-merge E2E-01/12/13 passed on the production setup (Oct 19).</t>
-  </si>
-  <si>
-    <t>None</t>
   </si>
 </sst>
 </file>
@@ -2237,7 +2234,7 @@
         <v>59</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="H24" s="29" t="s">
         <v>152</v>

</xml_diff>